<commit_message>
Update for Claude-based analysis, current as of this date.
Analysis performed through late-April 2026. This is up to date for pre-IPAC (not final IPAC proceedings), and the pre-tech note.
</commit_message>
<xml_diff>
--- a/Magnet_Studies/Data_Analysis/Cleanup_Claude/Materials_Arrangements.xlsx
+++ b/Magnet_Studies/Data_Analysis/Cleanup_Claude/Materials_Arrangements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryanmb/Documents/LDRD/Data_Plots/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryanmb/Documents/LDRD/Claude_Analysis1/Cleanup_Claude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0278D0F7-4C7B-9E4E-94F0-7C2F04E94CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C40C0B-CBAF-E549-8B3F-33C5E511E024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{365E0260-CCBB-4E43-809C-DC12287A7B21}"/>
+    <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{365E0260-CCBB-4E43-809C-DC12287A7B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Tunnel - Y Materials" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="137">
   <si>
     <t>Plate ID</t>
   </si>
@@ -267,13 +267,196 @@
   </si>
   <si>
     <t>Beta</t>
+  </si>
+  <si>
+    <t>n-1</t>
+  </si>
+  <si>
+    <t>n-2</t>
+  </si>
+  <si>
+    <t>n-3</t>
+  </si>
+  <si>
+    <t>n-5</t>
+  </si>
+  <si>
+    <t>n-7</t>
+  </si>
+  <si>
+    <t>n-13</t>
+  </si>
+  <si>
+    <t>n-14</t>
+  </si>
+  <si>
+    <t>n-21</t>
+  </si>
+  <si>
+    <t>n-22</t>
+  </si>
+  <si>
+    <t>n-23</t>
+  </si>
+  <si>
+    <t>n-25</t>
+  </si>
+  <si>
+    <t>n-26</t>
+  </si>
+  <si>
+    <t>n-27</t>
+  </si>
+  <si>
+    <t>n-28</t>
+  </si>
+  <si>
+    <t>n-29</t>
+  </si>
+  <si>
+    <t>n-30</t>
+  </si>
+  <si>
+    <t>n-31</t>
+  </si>
+  <si>
+    <t>n-32</t>
+  </si>
+  <si>
+    <t>n-33</t>
+  </si>
+  <si>
+    <t>n-34</t>
+  </si>
+  <si>
+    <t>n-35</t>
+  </si>
+  <si>
+    <t>n-36</t>
+  </si>
+  <si>
+    <t>n-38</t>
+  </si>
+  <si>
+    <t>n-40</t>
+  </si>
+  <si>
+    <t>s-8</t>
+  </si>
+  <si>
+    <t>s-9</t>
+  </si>
+  <si>
+    <t>s-11</t>
+  </si>
+  <si>
+    <t>s-19</t>
+  </si>
+  <si>
+    <t>s-21</t>
+  </si>
+  <si>
+    <t>s-22</t>
+  </si>
+  <si>
+    <t>s-23</t>
+  </si>
+  <si>
+    <t>s-24</t>
+  </si>
+  <si>
+    <t>s-25</t>
+  </si>
+  <si>
+    <t>s-26</t>
+  </si>
+  <si>
+    <t>s-27</t>
+  </si>
+  <si>
+    <t>s-28</t>
+  </si>
+  <si>
+    <t>s-29</t>
+  </si>
+  <si>
+    <t>s-30</t>
+  </si>
+  <si>
+    <t>s-31</t>
+  </si>
+  <si>
+    <t>s-32</t>
+  </si>
+  <si>
+    <t>s-33</t>
+  </si>
+  <si>
+    <t>s-34</t>
+  </si>
+  <si>
+    <t>s-35</t>
+  </si>
+  <si>
+    <t>s-36</t>
+  </si>
+  <si>
+    <t>s-37</t>
+  </si>
+  <si>
+    <t>s-38</t>
+  </si>
+  <si>
+    <t>s-39</t>
+  </si>
+  <si>
+    <t>s-40</t>
+  </si>
+  <si>
+    <t>y-8</t>
+  </si>
+  <si>
+    <t>N52SH</t>
+  </si>
+  <si>
+    <t>SmCo35</t>
+  </si>
+  <si>
+    <t>N42EH</t>
+  </si>
+  <si>
+    <t>SmCo33H</t>
+  </si>
+  <si>
+    <t>y-14</t>
+  </si>
+  <si>
+    <t>y-27</t>
+  </si>
+  <si>
+    <t>y-28</t>
+  </si>
+  <si>
+    <t>y-29</t>
+  </si>
+  <si>
+    <t>y-31</t>
+  </si>
+  <si>
+    <t>y-33</t>
+  </si>
+  <si>
+    <t>y-35</t>
+  </si>
+  <si>
+    <t>y-37</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -291,6 +474,12 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -315,10 +504,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1829,18 +2019,1170 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB7532DC-3C8D-E346-9037-F59C8BDDA03B}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659E7922-901F-C848-A475-A7D1E5EA4358}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>